<commit_message>
Se agregan capturas y BPMN a carpeta documentacion
</commit_message>
<xml_diff>
--- a/Datos/soporte.xlsx
+++ b/Datos/soporte.xlsx
@@ -526,6 +526,11 @@
           <t>Internet + Telefonía</t>
         </is>
       </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>TKT-0003</t>
+        </is>
+      </c>
       <c r="G3" t="inlineStr">
         <is>
           <t>20-07-2022</t>
@@ -628,14 +633,10 @@
       <c r="A2" t="n">
         <v>1090762400</v>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>CLI-0001</t>
-        </is>
-      </c>
+      <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr">
         <is>
-          <t>TICKET_GENERADO</t>
+          <t>FALLIDO</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -643,22 +644,22 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Otro problema</t>
+          <t>Conectividad (sin internet)</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>jemperador@outlook.com</t>
+          <t>tupad_prueba@tup.com</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>TKT-0002</t>
+          <t>TKT-0003</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>06-06-2026 11:15</t>
+          <t>06-06-2026 22:05</t>
         </is>
       </c>
     </row>
@@ -673,7 +674,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:H47"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="13.5703125" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -1177,6 +1178,874 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="n">
+        <v>1090762400</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>06-06-2026 21:32</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>CANCELADO</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>FALLIDO</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="n">
+        <v>1090762400</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>06-06-2026 21:34</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>INICIO_SESION</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>EXITOSO</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="n">
+        <v>1090762400</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>CLI-0001</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>06-06-2026 21:35</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>NUMERO_VALIDADO</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>EXITOSO</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="n">
+        <v>1090762400</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>CLI-0001</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>06-06-2026 21:36</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>CATEGORIA_SELECCIONADA</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Categoría: Conectividad (sin internet)</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>EXITOSO</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="n">
+        <v>1090762400</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>CLI-0001</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>06-06-2026 21:36</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>SOLUCION_MOSTRADA</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Categoría: Conectividad (sin internet)</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>EXITOSO</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="n">
+        <v>1090762400</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>CLI-0001</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>06-06-2026 21:36</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>PROBLEMA_RESUELTO</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>EXITOSO</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="n">
+        <v>1090762400</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>CLI-0001</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>06-06-2026 21:41</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>TIMEOUT</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>FALLIDO</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="n">
+        <v>1090762400</v>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>06-06-2026 21:41</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>INICIO_SESION</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>EXITOSO</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="n">
+        <v>1090762400</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>CLI-0002</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>06-06-2026 21:41</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>NUMERO_VALIDADO</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>EXITOSO</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="n">
+        <v>1090762400</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>CLI-0002</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>06-06-2026 21:41</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>CATEGORIA_SELECCIONADA</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Categoría: Conectividad (sin internet)</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>EXITOSO</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" t="n">
+        <v>1090762400</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>CLI-0002</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>06-06-2026 21:41</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>SOLUCION_MOSTRADA</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Categoría: Conectividad (sin internet)</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>EXITOSO</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" t="n">
+        <v>1090762400</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>CLI-0002</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>06-06-2026 21:42</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>EMAIL_REGISTRADO</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Email: tupad_prueba@tup.com</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>EXITOSO</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" t="n">
+        <v>1090762400</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>CLI-0002</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>06-06-2026 21:42</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>TICKET_GENERADO</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Categoría: Conectividad (sin internet)</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>EXITOSO</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>TKT-0003</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" t="n">
+        <v>1090762400</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>CLI-0002</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>06-06-2026 21:47</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>TIMEOUT</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>FALLIDO</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" t="n">
+        <v>1090762400</v>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>06-06-2026 21:48</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>INICIO_SESION</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>EXITOSO</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" t="n">
+        <v>1090762400</v>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>06-06-2026 21:49</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>NUMERO_INVALIDO</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>No encontrado en BD: CLI-0008. Intento 1</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>FALLIDO</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" t="n">
+        <v>1090762400</v>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>CLI-0003</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>06-06-2026 21:49</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>NUMERO_VALIDADO</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>EXITOSO</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" t="n">
+        <v>1090762400</v>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>CLI-0003</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>06-06-2026 21:49</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>CANCELADO</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>FALLIDO</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" t="n">
+        <v>1090762400</v>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>06-06-2026 21:50</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>INICIO_SESION</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>EXITOSO</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" t="n">
+        <v>1090762400</v>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>06-06-2026 21:50</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>NUMERO_INVALIDO</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>No encontrado en BD: CLI-0008. Intento 1</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>FALLIDO</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" t="n">
+        <v>1090762400</v>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>06-06-2026 21:50</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>NUMERO_INVALIDO</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>No encontrado en BD: CLI-0008. Intento 2</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>FALLIDO</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" t="n">
+        <v>1090762400</v>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>06-06-2026 21:50</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>NUMERO_INVALIDO</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>No encontrado en BD: CLI-0008. Intento 3</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>FALLIDO</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" t="n">
+        <v>1090762400</v>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>06-06-2026 21:52</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>INICIO_SESION</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>EXITOSO</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" t="n">
+        <v>1090762400</v>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>06-06-2026 21:52</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>NUMERO_INVALIDO</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Formato inválido: 0008. Intento 1</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>FALLIDO</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" t="n">
+        <v>1090762400</v>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>06-06-2026 21:56</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>TIMEOUT</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>FALLIDO</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" t="n">
+        <v>1090762400</v>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>06-06-2026 21:56</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>INICIO_SESION</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>EXITOSO</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" t="n">
+        <v>1090762400</v>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>CLI-0003</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>06-06-2026 21:56</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>NUMERO_VALIDADO</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>EXITOSO</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" t="n">
+        <v>1090762400</v>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>CLI-0003</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>06-06-2026 21:58</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>CATEGORIA_SELECCIONADA</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Categoría: Conectividad (sin internet)</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>EXITOSO</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" t="n">
+        <v>1090762400</v>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>CLI-0003</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>06-06-2026 21:58</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>SOLUCION_MOSTRADA</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Categoría: Conectividad (sin internet)</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>EXITOSO</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" t="n">
+        <v>1090762400</v>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>CLI-0003</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>06-06-2026 22:04</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>TIMEOUT</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>FALLIDO</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" t="n">
+        <v>1090762400</v>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>06-06-2026 22:05</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>CANCELADO</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>FALLIDO</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Merge (#3) from JEmperador
 - Se agregan capturas de bot
 - Se agrega captura de BPMN
 - Se agrega archivo drawio de BPMN
</commit_message>
<xml_diff>
--- a/Datos/soporte.xlsx
+++ b/Datos/soporte.xlsx
@@ -526,6 +526,11 @@
           <t>Internet + Telefonía</t>
         </is>
       </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>TKT-0003</t>
+        </is>
+      </c>
       <c r="G3" t="inlineStr">
         <is>
           <t>20-07-2022</t>
@@ -628,14 +633,10 @@
       <c r="A2" t="n">
         <v>1090762400</v>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>CLI-0001</t>
-        </is>
-      </c>
+      <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr">
         <is>
-          <t>TICKET_GENERADO</t>
+          <t>FALLIDO</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -643,22 +644,22 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Otro problema</t>
+          <t>Conectividad (sin internet)</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>jemperador@outlook.com</t>
+          <t>tupad_prueba@tup.com</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>TKT-0002</t>
+          <t>TKT-0003</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>06-06-2026 11:15</t>
+          <t>06-06-2026 22:05</t>
         </is>
       </c>
     </row>
@@ -673,7 +674,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:H47"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="13.5703125" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -1177,6 +1178,874 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="n">
+        <v>1090762400</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>06-06-2026 21:32</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>CANCELADO</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>FALLIDO</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="n">
+        <v>1090762400</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>06-06-2026 21:34</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>INICIO_SESION</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>EXITOSO</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="n">
+        <v>1090762400</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>CLI-0001</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>06-06-2026 21:35</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>NUMERO_VALIDADO</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>EXITOSO</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="n">
+        <v>1090762400</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>CLI-0001</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>06-06-2026 21:36</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>CATEGORIA_SELECCIONADA</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Categoría: Conectividad (sin internet)</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>EXITOSO</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="n">
+        <v>1090762400</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>CLI-0001</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>06-06-2026 21:36</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>SOLUCION_MOSTRADA</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Categoría: Conectividad (sin internet)</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>EXITOSO</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="n">
+        <v>1090762400</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>CLI-0001</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>06-06-2026 21:36</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>PROBLEMA_RESUELTO</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>EXITOSO</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="n">
+        <v>1090762400</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>CLI-0001</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>06-06-2026 21:41</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>TIMEOUT</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>FALLIDO</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="n">
+        <v>1090762400</v>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>06-06-2026 21:41</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>INICIO_SESION</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>EXITOSO</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="n">
+        <v>1090762400</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>CLI-0002</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>06-06-2026 21:41</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>NUMERO_VALIDADO</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>EXITOSO</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="n">
+        <v>1090762400</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>CLI-0002</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>06-06-2026 21:41</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>CATEGORIA_SELECCIONADA</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Categoría: Conectividad (sin internet)</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>EXITOSO</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" t="n">
+        <v>1090762400</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>CLI-0002</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>06-06-2026 21:41</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>SOLUCION_MOSTRADA</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Categoría: Conectividad (sin internet)</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>EXITOSO</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" t="n">
+        <v>1090762400</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>CLI-0002</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>06-06-2026 21:42</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>EMAIL_REGISTRADO</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Email: tupad_prueba@tup.com</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>EXITOSO</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" t="n">
+        <v>1090762400</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>CLI-0002</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>06-06-2026 21:42</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>TICKET_GENERADO</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Categoría: Conectividad (sin internet)</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>EXITOSO</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>TKT-0003</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" t="n">
+        <v>1090762400</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>CLI-0002</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>06-06-2026 21:47</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>TIMEOUT</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>FALLIDO</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" t="n">
+        <v>1090762400</v>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>06-06-2026 21:48</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>INICIO_SESION</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>EXITOSO</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" t="n">
+        <v>1090762400</v>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>06-06-2026 21:49</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>NUMERO_INVALIDO</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>No encontrado en BD: CLI-0008. Intento 1</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>FALLIDO</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" t="n">
+        <v>1090762400</v>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>CLI-0003</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>06-06-2026 21:49</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>NUMERO_VALIDADO</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>EXITOSO</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" t="n">
+        <v>1090762400</v>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>CLI-0003</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>06-06-2026 21:49</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>CANCELADO</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>FALLIDO</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" t="n">
+        <v>1090762400</v>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>06-06-2026 21:50</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>INICIO_SESION</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>EXITOSO</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" t="n">
+        <v>1090762400</v>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>06-06-2026 21:50</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>NUMERO_INVALIDO</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>No encontrado en BD: CLI-0008. Intento 1</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>FALLIDO</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" t="n">
+        <v>1090762400</v>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>06-06-2026 21:50</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>NUMERO_INVALIDO</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>No encontrado en BD: CLI-0008. Intento 2</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>FALLIDO</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" t="n">
+        <v>1090762400</v>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>06-06-2026 21:50</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>NUMERO_INVALIDO</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>No encontrado en BD: CLI-0008. Intento 3</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>FALLIDO</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" t="n">
+        <v>1090762400</v>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>06-06-2026 21:52</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>INICIO_SESION</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>EXITOSO</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" t="n">
+        <v>1090762400</v>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>06-06-2026 21:52</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>NUMERO_INVALIDO</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Formato inválido: 0008. Intento 1</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>FALLIDO</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" t="n">
+        <v>1090762400</v>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>06-06-2026 21:56</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>TIMEOUT</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>FALLIDO</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" t="n">
+        <v>1090762400</v>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>06-06-2026 21:56</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>INICIO_SESION</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>EXITOSO</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" t="n">
+        <v>1090762400</v>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>CLI-0003</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>06-06-2026 21:56</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>NUMERO_VALIDADO</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>EXITOSO</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" t="n">
+        <v>1090762400</v>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>CLI-0003</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>06-06-2026 21:58</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>CATEGORIA_SELECCIONADA</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Categoría: Conectividad (sin internet)</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>EXITOSO</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" t="n">
+        <v>1090762400</v>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>CLI-0003</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>06-06-2026 21:58</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>SOLUCION_MOSTRADA</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Categoría: Conectividad (sin internet)</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>EXITOSO</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" t="n">
+        <v>1090762400</v>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>CLI-0003</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>06-06-2026 22:04</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>TIMEOUT</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>FALLIDO</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" t="n">
+        <v>1090762400</v>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>06-06-2026 22:05</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>CANCELADO</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>FALLIDO</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>